<commit_message>
pcb: LCSC BOM with quantities per board
The upload file now carries the number of parts for one board (159 parts, 66 lines),
not rounded to LCSC minimum orders and without spares; --boards and --spare-rate
give other quantities. The full BOM keeps the LCSC minimum, multiple and the
rounded order cost for 1 board (USD 59.92) and 5 boards (USD 148.58).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/PCB_V1/BOM_LCSC_v22.xlsx
+++ b/pcb/PCB_V1/BOM_LCSC_v22.xlsx
@@ -151,7 +151,7 @@
     </row>
     <row r="2">
       <c r="A2" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -181,7 +181,7 @@
     </row>
     <row r="3">
       <c r="A3" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -211,7 +211,7 @@
     </row>
     <row r="4">
       <c r="A4" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -241,7 +241,7 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -271,7 +271,7 @@
     </row>
     <row r="6">
       <c r="A6" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -301,7 +301,7 @@
     </row>
     <row r="7">
       <c r="A7" s="4">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -331,7 +331,7 @@
     </row>
     <row r="8">
       <c r="A8" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -361,7 +361,7 @@
     </row>
     <row r="9">
       <c r="A9" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -391,7 +391,7 @@
     </row>
     <row r="10">
       <c r="A10" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -421,7 +421,7 @@
     </row>
     <row r="11">
       <c r="A11" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -451,7 +451,7 @@
     </row>
     <row r="12">
       <c r="A12" s="4">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
     </row>
     <row r="13">
       <c r="A13" s="4">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -511,7 +511,7 @@
     </row>
     <row r="14">
       <c r="A14" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
     </row>
     <row r="15">
       <c r="A15" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -571,7 +571,7 @@
     </row>
     <row r="16">
       <c r="A16" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
     </row>
     <row r="17">
       <c r="A17" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -631,7 +631,7 @@
     </row>
     <row r="18">
       <c r="A18" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10u FXL0630-100-M L_Changjiang_FXL0630</t>
+          <t xml:space="preserve">cjiang FXL0630-100-M</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -661,7 +661,7 @@
     </row>
     <row r="19">
       <c r="A19" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">47u SRP1770TA-470M L_Bourns_SRP1770TA_16.9x16.9mm</t>
+          <t xml:space="preserve">Bourns SRP1770TA-470M</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
     </row>
     <row r="20">
       <c r="A20" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">47u SRP1265A-470M L_Bourns_SRP1265A</t>
+          <t xml:space="preserve">Bourns SRP1265A-470M</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
     </row>
     <row r="21">
       <c r="A21" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22u PSPMAA0604-220M L_Changjiang_FXL0630</t>
+          <t xml:space="preserve">PROD Tech PSPMAA0604-220M-ANP</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -751,7 +751,7 @@
     </row>
     <row r="22">
       <c r="A22" s="4">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -781,7 +781,7 @@
     </row>
     <row r="23">
       <c r="A23" s="4">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     </row>
     <row r="24">
       <c r="A24" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
     </row>
     <row r="25">
       <c r="A25" s="4">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
     </row>
     <row r="28">
       <c r="A28" s="4">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
     </row>
     <row r="29">
       <c r="A29" s="4">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -991,7 +991,7 @@
     </row>
     <row r="30">
       <c r="A30" s="4">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="31">
       <c r="A31" s="4">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -1051,7 +1051,7 @@
     </row>
     <row r="32">
       <c r="A32" s="4">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
     </row>
     <row r="33">
       <c r="A33" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="34">
       <c r="A34" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
     </row>
     <row r="35">
       <c r="A35" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="36">
       <c r="A36" s="4">
-        <v>100</v>
+        <v>7</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
     </row>
     <row r="37">
       <c r="A37" s="4">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
     </row>
     <row r="38">
       <c r="A38" s="4">
-        <v>200</v>
+        <v>19</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
     </row>
     <row r="39">
       <c r="A39" s="4">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="40">
       <c r="A40" s="4">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
     </row>
     <row r="41">
       <c r="A41" s="4">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
     </row>
     <row r="42">
       <c r="A42" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
     </row>
     <row r="43">
       <c r="A43" s="4">
-        <v>100</v>
+        <v>3</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
     </row>
     <row r="44">
       <c r="A44" s="4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
     </row>
     <row r="45">
       <c r="A45" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
     </row>
     <row r="46">
       <c r="A46" s="4">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
     </row>
     <row r="47">
       <c r="A47" s="4">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="48">
       <c r="A48" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
     </row>
     <row r="49">
       <c r="A49" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -1591,7 +1591,7 @@
     </row>
     <row r="50">
       <c r="A50" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="51">
       <c r="A51" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="52">
       <c r="A52" s="4">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
     </row>
     <row r="53">
       <c r="A53" s="4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="54">
       <c r="A54" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
     </row>
     <row r="55">
       <c r="A55" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
     </row>
     <row r="56">
       <c r="A56" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
     </row>
     <row r="57">
       <c r="A57" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
     </row>
     <row r="58">
       <c r="A58" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
@@ -1861,7 +1861,7 @@
     </row>
     <row r="59">
       <c r="A59" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
@@ -1891,7 +1891,7 @@
     </row>
     <row r="60">
       <c r="A60" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
     </row>
     <row r="61">
       <c r="A61" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
     </row>
     <row r="62">
       <c r="A62" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
     </row>
     <row r="63">
       <c r="A63" s="4">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
@@ -2011,7 +2011,7 @@
     </row>
     <row r="64">
       <c r="A64" s="4">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
@@ -2041,7 +2041,7 @@
     </row>
     <row r="65">
       <c r="A65" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
@@ -2071,7 +2071,7 @@
     </row>
     <row r="66">
       <c r="A66" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
@@ -2101,7 +2101,7 @@
     </row>
     <row r="67">
       <c r="A67" s="4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
@@ -2157,12 +2157,11 @@
     <col min="17" max="17" width="10" customWidth="1"/>
     <col min="18" max="18" width="10" customWidth="1"/>
     <col min="19" max="19" width="10" customWidth="1"/>
-    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="20" max="20" width="10" customWidth="1"/>
     <col min="21" max="21" width="10" customWidth="1"/>
     <col min="22" max="22" width="10" customWidth="1"/>
-    <col min="23" max="23" width="10" customWidth="1"/>
-    <col min="24" max="24" width="34" customWidth="1"/>
-    <col min="25" max="25" width="60" customWidth="1"/>
+    <col min="23" max="23" width="34" customWidth="1"/>
+    <col min="24" max="24" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2258,35 +2257,30 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needed 5 boards</t>
+          <t xml:space="preserve">Order qty 5 boards</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spares and MOQ surplus</t>
+          <t xml:space="preserve">Unit USD 5 boards</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order qty 5 boards</t>
+          <t xml:space="preserve">Order USD 5 boards</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit USD 5 boards</t>
+          <t xml:space="preserve">Qty in BOM_LCSC file</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order USD 5 boards</t>
+          <t xml:space="preserve">LCSC page</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LCSC page</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes</t>
         </is>
@@ -2364,34 +2358,27 @@
       <c r="Q2" s="3">
         <v>0.1742</v>
       </c>
-      <c r="R2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8710</t>
-        </is>
+      <c r="R2" s="3">
+        <v>0.871</v>
       </c>
       <c r="S2" s="4">
         <v>5</v>
       </c>
-      <c r="T2" s="4">
-        <v>5</v>
-      </c>
-      <c r="U2" s="4">
-        <v>10</v>
-      </c>
-      <c r="V2" s="3">
+      <c r="T2" s="3">
         <v>0.1742</v>
       </c>
-      <c r="W2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7420</t>
-        </is>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="U2" s="3">
+        <v>0.871</v>
+      </c>
+      <c r="V2" s="4">
+        <v>1</v>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C191884.html</t>
         </is>
       </c>
-      <c r="Y2" s="2"/>
+      <c r="X2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" s="4">
@@ -2465,34 +2452,27 @@
       <c r="Q3" s="3">
         <v>3.7644</v>
       </c>
-      <c r="R3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.7644</t>
-        </is>
+      <c r="R3" s="3">
+        <v>3.7644</v>
       </c>
       <c r="S3" s="4">
         <v>5</v>
       </c>
-      <c r="T3" s="4">
-        <v>1</v>
-      </c>
-      <c r="U3" s="4">
-        <v>6</v>
-      </c>
-      <c r="V3" s="3">
+      <c r="T3" s="3">
         <v>3.7644</v>
       </c>
-      <c r="W3" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22.5864</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
+      <c r="U3" s="3">
+        <v>18.822</v>
+      </c>
+      <c r="V3" s="4">
+        <v>1</v>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C701341.html</t>
         </is>
       </c>
-      <c r="Y3" s="2"/>
+      <c r="X3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" s="4">
@@ -2566,34 +2546,27 @@
       <c r="Q4" s="3">
         <v>0.6138</v>
       </c>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6138</t>
-        </is>
+      <c r="R4" s="3">
+        <v>0.6138</v>
       </c>
       <c r="S4" s="4">
         <v>5</v>
       </c>
-      <c r="T4" s="4">
-        <v>1</v>
-      </c>
-      <c r="U4" s="4">
-        <v>6</v>
-      </c>
-      <c r="V4" s="3">
+      <c r="T4" s="3">
         <v>0.6138</v>
       </c>
-      <c r="W4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.6828</t>
+      <c r="U4" s="3">
+        <v>3.069</v>
+      </c>
+      <c r="V4" s="4">
+        <v>1</v>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C7440.html</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C7440.html</t>
-        </is>
-      </c>
-      <c r="Y4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">RTC, I2C 0x51; replaces DS3231MZ+TRL (firmware auto-detects either)</t>
         </is>
@@ -2671,34 +2644,27 @@
       <c r="Q5" s="3">
         <v>0.2783</v>
       </c>
-      <c r="R5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3915</t>
-        </is>
+      <c r="R5" s="3">
+        <v>1.3915</v>
       </c>
       <c r="S5" s="4">
         <v>5</v>
       </c>
-      <c r="T5" s="4">
-        <v>5</v>
-      </c>
-      <c r="U5" s="4">
-        <v>10</v>
-      </c>
-      <c r="V5" s="3">
+      <c r="T5" s="3">
         <v>0.2783</v>
       </c>
-      <c r="W5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.7830</t>
-        </is>
-      </c>
-      <c r="X5" s="2" t="inlineStr">
+      <c r="U5" s="3">
+        <v>1.3915</v>
+      </c>
+      <c r="V5" s="4">
+        <v>1</v>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C185857.html</t>
         </is>
       </c>
-      <c r="Y5" s="2"/>
+      <c r="X5" s="2"/>
     </row>
     <row r="6">
       <c r="A6" s="4">
@@ -2772,34 +2738,27 @@
       <c r="Q6" s="3">
         <v>0.0496</v>
       </c>
-      <c r="R6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4960</t>
-        </is>
+      <c r="R6" s="3">
+        <v>0.496</v>
       </c>
       <c r="S6" s="4">
-        <v>5</v>
-      </c>
-      <c r="T6" s="4">
-        <v>5</v>
-      </c>
-      <c r="U6" s="4">
         <v>10</v>
       </c>
-      <c r="V6" s="3">
+      <c r="T6" s="3">
         <v>0.0496</v>
       </c>
-      <c r="W6" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4960</t>
-        </is>
-      </c>
-      <c r="X6" s="2" t="inlineStr">
+      <c r="U6" s="3">
+        <v>0.496</v>
+      </c>
+      <c r="V6" s="4">
+        <v>1</v>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C7666.html</t>
         </is>
       </c>
-      <c r="Y6" s="2"/>
+      <c r="X6" s="2"/>
     </row>
     <row r="7">
       <c r="A7" s="4">
@@ -2873,34 +2832,27 @@
       <c r="Q7" s="3">
         <v>0.9392</v>
       </c>
-      <c r="R7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.8784</t>
-        </is>
+      <c r="R7" s="3">
+        <v>1.8784</v>
       </c>
       <c r="S7" s="4">
         <v>10</v>
       </c>
-      <c r="T7" s="4">
-        <v>1</v>
-      </c>
-      <c r="U7" s="4">
-        <v>11</v>
-      </c>
-      <c r="V7" s="3">
+      <c r="T7" s="3">
         <v>0.7339</v>
       </c>
-      <c r="W7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8.0729</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="U7" s="3">
+        <v>7.339</v>
+      </c>
+      <c r="V7" s="4">
+        <v>2</v>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C3192318.html</t>
         </is>
       </c>
-      <c r="Y7" s="2"/>
+      <c r="X7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" s="4">
@@ -2974,34 +2926,27 @@
       <c r="Q8" s="3">
         <v>0.8159</v>
       </c>
-      <c r="R8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8159</t>
-        </is>
+      <c r="R8" s="3">
+        <v>0.8159</v>
       </c>
       <c r="S8" s="4">
         <v>5</v>
       </c>
-      <c r="T8" s="4">
-        <v>1</v>
-      </c>
-      <c r="U8" s="4">
-        <v>6</v>
-      </c>
-      <c r="V8" s="3">
+      <c r="T8" s="3">
         <v>0.8159</v>
       </c>
-      <c r="W8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.8954</t>
-        </is>
-      </c>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="U8" s="3">
+        <v>4.0795</v>
+      </c>
+      <c r="V8" s="4">
+        <v>1</v>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C190006.html</t>
         </is>
       </c>
-      <c r="Y8" s="2"/>
+      <c r="X8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" s="4">
@@ -3075,34 +3020,27 @@
       <c r="Q9" s="3">
         <v>0.0853</v>
       </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4265</t>
-        </is>
+      <c r="R9" s="3">
+        <v>0.4265</v>
       </c>
       <c r="S9" s="4">
         <v>10</v>
       </c>
-      <c r="T9" s="4">
-        <v>5</v>
-      </c>
-      <c r="U9" s="4">
-        <v>15</v>
-      </c>
-      <c r="V9" s="3">
+      <c r="T9" s="3">
         <v>0.0853</v>
       </c>
-      <c r="W9" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2795</t>
-        </is>
-      </c>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="U9" s="3">
+        <v>0.853</v>
+      </c>
+      <c r="V9" s="4">
+        <v>2</v>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C20917.html</t>
         </is>
       </c>
-      <c r="Y9" s="2"/>
+      <c r="X9" s="2"/>
     </row>
     <row r="10">
       <c r="A10" s="4">
@@ -3176,34 +3114,27 @@
       <c r="Q10" s="3">
         <v>0.1356</v>
       </c>
-      <c r="R10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6780</t>
-        </is>
+      <c r="R10" s="3">
+        <v>0.678</v>
       </c>
       <c r="S10" s="4">
         <v>5</v>
       </c>
-      <c r="T10" s="4">
-        <v>5</v>
-      </c>
-      <c r="U10" s="4">
-        <v>10</v>
-      </c>
-      <c r="V10" s="3">
+      <c r="T10" s="3">
         <v>0.1356</v>
       </c>
-      <c r="W10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3560</t>
-        </is>
-      </c>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="U10" s="3">
+        <v>0.678</v>
+      </c>
+      <c r="V10" s="4">
+        <v>1</v>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C37130.html</t>
         </is>
       </c>
-      <c r="Y10" s="2"/>
+      <c r="X10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" s="4">
@@ -3277,34 +3208,27 @@
       <c r="Q11" s="3">
         <v>0.7717</v>
       </c>
-      <c r="R11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7717</t>
-        </is>
+      <c r="R11" s="3">
+        <v>0.7717</v>
       </c>
       <c r="S11" s="4">
         <v>5</v>
       </c>
-      <c r="T11" s="4">
-        <v>1</v>
-      </c>
-      <c r="U11" s="4">
-        <v>6</v>
-      </c>
-      <c r="V11" s="3">
+      <c r="T11" s="3">
         <v>0.7717</v>
       </c>
-      <c r="W11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.6302</t>
-        </is>
-      </c>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="U11" s="3">
+        <v>3.8585</v>
+      </c>
+      <c r="V11" s="4">
+        <v>1</v>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C145537.html</t>
         </is>
       </c>
-      <c r="Y11" s="2"/>
+      <c r="X11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" s="4">
@@ -3378,34 +3302,27 @@
       <c r="Q12" s="3">
         <v>0.4343</v>
       </c>
-      <c r="R12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8686</t>
-        </is>
+      <c r="R12" s="3">
+        <v>0.8686</v>
       </c>
       <c r="S12" s="4">
         <v>10</v>
       </c>
-      <c r="T12" s="4">
-        <v>1</v>
-      </c>
-      <c r="U12" s="4">
-        <v>11</v>
-      </c>
-      <c r="V12" s="3">
+      <c r="T12" s="3">
         <v>0.3853</v>
       </c>
-      <c r="W12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.2383</t>
+      <c r="U12" s="3">
+        <v>3.853</v>
+      </c>
+      <c r="V12" s="4">
+        <v>2</v>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C485687.html</t>
         </is>
       </c>
       <c r="X12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C485687.html</t>
-        </is>
-      </c>
-      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">100 V DPAK; replaces CSD19534Q5A and CSD19538Q3A</t>
         </is>
@@ -3483,34 +3400,27 @@
       <c r="Q13" s="3">
         <v>0.1131</v>
       </c>
-      <c r="R13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.5655</t>
-        </is>
+      <c r="R13" s="3">
+        <v>0.5655</v>
       </c>
       <c r="S13" s="4">
         <v>20</v>
       </c>
-      <c r="T13" s="4">
-        <v>5</v>
-      </c>
-      <c r="U13" s="4">
-        <v>25</v>
-      </c>
-      <c r="V13" s="3">
+      <c r="T13" s="3">
         <v>0.1131</v>
       </c>
-      <c r="W13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.8275</t>
+      <c r="U13" s="3">
+        <v>2.262</v>
+      </c>
+      <c r="V13" s="4">
+        <v>4</v>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C5350871.html</t>
         </is>
       </c>
       <c r="X13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C5350871.html</t>
-        </is>
-      </c>
-      <c r="Y13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">second source: the original part is out of stock; TI TPD2E2U06DCKR C1855726 has 0 in stock</t>
         </is>
@@ -3588,34 +3498,27 @@
       <c r="Q14" s="3">
         <v>0.0301</v>
       </c>
-      <c r="R14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6020</t>
-        </is>
+      <c r="R14" s="3">
+        <v>0.602</v>
       </c>
       <c r="S14" s="4">
-        <v>5</v>
-      </c>
-      <c r="T14" s="4">
-        <v>15</v>
-      </c>
-      <c r="U14" s="4">
         <v>20</v>
       </c>
-      <c r="V14" s="3">
+      <c r="T14" s="3">
         <v>0.0301</v>
       </c>
-      <c r="W14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6020</t>
+      <c r="U14" s="3">
+        <v>0.602</v>
+      </c>
+      <c r="V14" s="4">
+        <v>1</v>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C68970.html</t>
         </is>
       </c>
       <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C68970.html</t>
-        </is>
-      </c>
-      <c r="Y14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">v0.21 RTC OR: low-leakage silicon common cathode diode; room-temperature specification only for selected JSCJ part</t>
         </is>
@@ -3693,34 +3596,27 @@
       <c r="Q15" s="3">
         <v>0.3327</v>
       </c>
-      <c r="R15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6635</t>
-        </is>
+      <c r="R15" s="3">
+        <v>1.6635</v>
       </c>
       <c r="S15" s="4">
         <v>10</v>
       </c>
-      <c r="T15" s="4">
-        <v>5</v>
-      </c>
-      <c r="U15" s="4">
-        <v>15</v>
-      </c>
-      <c r="V15" s="3">
+      <c r="T15" s="3">
         <v>0.3327</v>
       </c>
-      <c r="W15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.9905</t>
-        </is>
-      </c>
-      <c r="X15" s="2" t="inlineStr">
+      <c r="U15" s="3">
+        <v>3.327</v>
+      </c>
+      <c r="V15" s="4">
+        <v>2</v>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C35722.html</t>
         </is>
       </c>
-      <c r="Y15" s="2"/>
+      <c r="X15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" s="4">
@@ -3794,34 +3690,27 @@
       <c r="Q16" s="3">
         <v>0.1036</v>
       </c>
-      <c r="R16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.5180</t>
-        </is>
+      <c r="R16" s="3">
+        <v>0.518</v>
       </c>
       <c r="S16" s="4">
         <v>10</v>
       </c>
-      <c r="T16" s="4">
-        <v>5</v>
-      </c>
-      <c r="U16" s="4">
-        <v>15</v>
-      </c>
-      <c r="V16" s="3">
+      <c r="T16" s="3">
         <v>0.1036</v>
       </c>
-      <c r="W16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5540</t>
+      <c r="U16" s="3">
+        <v>1.036</v>
+      </c>
+      <c r="V16" s="4">
+        <v>2</v>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C515606.html</t>
         </is>
       </c>
       <c r="X16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C515606.html</t>
-        </is>
-      </c>
-      <c r="Y16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">D601 moved from SMBJ30A to the input TVS part</t>
         </is>
@@ -3899,34 +3788,27 @@
       <c r="Q17" s="3">
         <v>0.2871</v>
       </c>
-      <c r="R17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.4355</t>
-        </is>
+      <c r="R17" s="3">
+        <v>1.4355</v>
       </c>
       <c r="S17" s="4">
         <v>10</v>
       </c>
-      <c r="T17" s="4">
-        <v>5</v>
-      </c>
-      <c r="U17" s="4">
-        <v>15</v>
-      </c>
-      <c r="V17" s="3">
+      <c r="T17" s="3">
         <v>0.2871</v>
       </c>
-      <c r="W17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4.3065</t>
+      <c r="U17" s="3">
+        <v>2.871</v>
+      </c>
+      <c r="V17" s="4">
+        <v>2</v>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C46986.html</t>
         </is>
       </c>
       <c r="X17" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C46986.html</t>
-        </is>
-      </c>
-      <c r="Y17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">100 V 5 A TO-277A; replaces STPS5H100B and STPS2H100AFY</t>
         </is>
@@ -4004,34 +3886,27 @@
       <c r="Q18" s="3">
         <v>0.1695</v>
       </c>
-      <c r="R18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8475</t>
-        </is>
+      <c r="R18" s="3">
+        <v>0.8475</v>
       </c>
       <c r="S18" s="4">
         <v>5</v>
       </c>
-      <c r="T18" s="4">
-        <v>5</v>
-      </c>
-      <c r="U18" s="4">
-        <v>10</v>
-      </c>
-      <c r="V18" s="3">
+      <c r="T18" s="3">
         <v>0.1695</v>
       </c>
-      <c r="W18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6950</t>
+      <c r="U18" s="3">
+        <v>0.8475</v>
+      </c>
+      <c r="V18" s="4">
+        <v>1</v>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C167223.html</t>
         </is>
       </c>
       <c r="X18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C167223.html</t>
-        </is>
-      </c>
-      <c r="Y18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">10uH, DCR 68 mOhm max, Isat 4.9 A</t>
         </is>
@@ -4109,34 +3984,27 @@
       <c r="Q19" s="3">
         <v>2.9304</v>
       </c>
-      <c r="R19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.9304</t>
-        </is>
+      <c r="R19" s="3">
+        <v>2.9304</v>
       </c>
       <c r="S19" s="4">
         <v>5</v>
       </c>
-      <c r="T19" s="4">
-        <v>1</v>
-      </c>
-      <c r="U19" s="4">
-        <v>6</v>
-      </c>
-      <c r="V19" s="3">
+      <c r="T19" s="3">
         <v>2.9304</v>
       </c>
-      <c r="W19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17.5824</t>
-        </is>
-      </c>
-      <c r="X19" s="2" t="inlineStr">
+      <c r="U19" s="3">
+        <v>14.652</v>
+      </c>
+      <c r="V19" s="4">
+        <v>1</v>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C2041872.html</t>
         </is>
       </c>
-      <c r="Y19" s="2"/>
+      <c r="X19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" s="4">
@@ -4210,34 +4078,27 @@
       <c r="Q20" s="3">
         <v>1.1226</v>
       </c>
-      <c r="R20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.1226</t>
-        </is>
+      <c r="R20" s="3">
+        <v>1.1226</v>
       </c>
       <c r="S20" s="4">
         <v>5</v>
       </c>
-      <c r="T20" s="4">
-        <v>1</v>
-      </c>
-      <c r="U20" s="4">
-        <v>6</v>
-      </c>
-      <c r="V20" s="3">
+      <c r="T20" s="3">
         <v>1.1226</v>
       </c>
-      <c r="W20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.7356</t>
-        </is>
-      </c>
-      <c r="X20" s="2" t="inlineStr">
+      <c r="U20" s="3">
+        <v>5.613</v>
+      </c>
+      <c r="V20" s="4">
+        <v>1</v>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C840530.html</t>
         </is>
       </c>
-      <c r="Y20" s="2"/>
+      <c r="X20" s="2"/>
     </row>
     <row r="21">
       <c r="A21" s="4">
@@ -4311,34 +4172,27 @@
       <c r="Q21" s="3">
         <v>0.1242</v>
       </c>
-      <c r="R21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6210</t>
-        </is>
+      <c r="R21" s="3">
+        <v>0.621</v>
       </c>
       <c r="S21" s="4">
         <v>5</v>
       </c>
-      <c r="T21" s="4">
-        <v>5</v>
-      </c>
-      <c r="U21" s="4">
-        <v>10</v>
-      </c>
-      <c r="V21" s="3">
+      <c r="T21" s="3">
         <v>0.1242</v>
       </c>
-      <c r="W21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2420</t>
+      <c r="U21" s="3">
+        <v>0.621</v>
+      </c>
+      <c r="V21" s="4">
+        <v>1</v>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C53190553.html</t>
         </is>
       </c>
       <c r="X21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C53190553.html</t>
-        </is>
-      </c>
-      <c r="Y21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">22uH, DCR 130 mOhm max, Isat 5 A (L -30 %), Irms 3.2 A</t>
         </is>
@@ -4416,34 +4270,27 @@
       <c r="Q22" s="3">
         <v>0.3569</v>
       </c>
-      <c r="R22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7138</t>
-        </is>
+      <c r="R22" s="3">
+        <v>0.7138</v>
       </c>
       <c r="S22" s="4">
         <v>10</v>
       </c>
-      <c r="T22" s="4">
-        <v>1</v>
-      </c>
-      <c r="U22" s="4">
-        <v>11</v>
-      </c>
-      <c r="V22" s="3">
+      <c r="T22" s="3">
         <v>0.2814</v>
       </c>
-      <c r="W22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.0954</t>
+      <c r="U22" s="3">
+        <v>2.814</v>
+      </c>
+      <c r="V22" s="4">
+        <v>2</v>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C309062.html</t>
         </is>
       </c>
       <c r="X22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C309062.html</t>
-        </is>
-      </c>
-      <c r="Y22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">C101 and C910 now explicitly select the same 22uF/25V X7R 1210; both on 12V aux.</t>
         </is>
@@ -4521,34 +4368,27 @@
       <c r="Q23" s="3">
         <v>0.0085</v>
       </c>
-      <c r="R23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8500</t>
-        </is>
+      <c r="R23" s="3">
+        <v>0.85</v>
       </c>
       <c r="S23" s="4">
-        <v>50</v>
-      </c>
-      <c r="T23" s="4">
-        <v>50</v>
-      </c>
-      <c r="U23" s="4">
         <v>100</v>
       </c>
-      <c r="V23" s="3">
+      <c r="T23" s="3">
         <v>0.0085</v>
       </c>
-      <c r="W23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8500</t>
+      <c r="U23" s="3">
+        <v>0.85</v>
+      </c>
+      <c r="V23" s="4">
+        <v>10</v>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C1591.html</t>
         </is>
       </c>
       <c r="X23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C1591.html</t>
-        </is>
-      </c>
-      <c r="Y23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">100n 50V X7R 0603 for every 100n 0603 position</t>
         </is>
@@ -4626,34 +4466,27 @@
       <c r="Q24" s="3">
         <v>0.0824</v>
       </c>
-      <c r="R24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8240</t>
-        </is>
+      <c r="R24" s="3">
+        <v>0.824</v>
       </c>
       <c r="S24" s="4">
-        <v>15</v>
-      </c>
-      <c r="T24" s="4">
-        <v>5</v>
-      </c>
-      <c r="U24" s="4">
         <v>20</v>
       </c>
-      <c r="V24" s="3">
+      <c r="T24" s="3">
         <v>0.0824</v>
       </c>
-      <c r="W24" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.6480</t>
+      <c r="U24" s="3">
+        <v>1.648</v>
+      </c>
+      <c r="V24" s="4">
+        <v>3</v>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C29277.html</t>
         </is>
       </c>
       <c r="X24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C29277.html</t>
-        </is>
-      </c>
-      <c r="Y24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">22u 10V X5R 0805; ~9.9uF each at 3.3 V (Samsung curve)</t>
         </is>
@@ -4731,34 +4564,27 @@
       <c r="Q25" s="3">
         <v>0.0798</v>
       </c>
-      <c r="R25" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5960</t>
-        </is>
+      <c r="R25" s="3">
+        <v>1.596</v>
       </c>
       <c r="S25" s="4">
-        <v>10</v>
-      </c>
-      <c r="T25" s="4">
-        <v>10</v>
-      </c>
-      <c r="U25" s="4">
         <v>20</v>
       </c>
-      <c r="V25" s="3">
+      <c r="T25" s="3">
         <v>0.0798</v>
       </c>
-      <c r="W25" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.5960</t>
+      <c r="U25" s="3">
+        <v>1.596</v>
+      </c>
+      <c r="V25" s="4">
+        <v>2</v>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C15850.html</t>
         </is>
       </c>
       <c r="X25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C15850.html</t>
-        </is>
-      </c>
-      <c r="Y25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">10u 25V X5R 0805; C602 &gt;=1uF effective at 12.26 V (Samsung curve ~1.83uF typ.)</t>
         </is>
@@ -4836,34 +4662,27 @@
       <c r="Q26" s="3">
         <v>0.0178</v>
       </c>
-      <c r="R26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.1780</t>
-        </is>
+      <c r="R26" s="3">
+        <v>0.178</v>
       </c>
       <c r="S26" s="4">
         <v>10</v>
       </c>
-      <c r="T26" s="4">
-        <v>10</v>
-      </c>
-      <c r="U26" s="4">
-        <v>20</v>
-      </c>
-      <c r="V26" s="3">
+      <c r="T26" s="3">
         <v>0.0178</v>
       </c>
-      <c r="W26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3560</t>
+      <c r="U26" s="3">
+        <v>0.178</v>
+      </c>
+      <c r="V26" s="4">
+        <v>2</v>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C29936.html</t>
         </is>
       </c>
       <c r="X26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C29936.html</t>
-        </is>
-      </c>
-      <c r="Y26" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package; 1u 25V X7R 0603 (JLC basic C15849 has 50 in stock)</t>
         </is>
@@ -4941,34 +4760,27 @@
       <c r="Q27" s="3">
         <v>0.0159</v>
       </c>
-      <c r="R27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7950</t>
-        </is>
+      <c r="R27" s="3">
+        <v>0.795</v>
       </c>
       <c r="S27" s="4">
-        <v>5</v>
-      </c>
-      <c r="T27" s="4">
-        <v>45</v>
-      </c>
-      <c r="U27" s="4">
         <v>50</v>
       </c>
-      <c r="V27" s="3">
+      <c r="T27" s="3">
         <v>0.0159</v>
       </c>
-      <c r="W27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7950</t>
+      <c r="U27" s="3">
+        <v>0.795</v>
+      </c>
+      <c r="V27" s="4">
+        <v>1</v>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C1647.html</t>
         </is>
       </c>
       <c r="X27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C1647.html</t>
-        </is>
-      </c>
-      <c r="Y27" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">18p 50V C0G 0603; PCF8563 OSCI load, value to be trimmed on the prototype</t>
         </is>
@@ -5046,34 +4858,27 @@
       <c r="Q28" s="3">
         <v>0.2929</v>
       </c>
-      <c r="R28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.9290</t>
-        </is>
+      <c r="R28" s="3">
+        <v>2.929</v>
       </c>
       <c r="S28" s="4">
         <v>30</v>
       </c>
-      <c r="T28" s="4">
-        <v>5</v>
-      </c>
-      <c r="U28" s="4">
-        <v>35</v>
-      </c>
-      <c r="V28" s="3">
+      <c r="T28" s="3">
         <v>0.2929</v>
       </c>
-      <c r="W28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10.2515</t>
+      <c r="U28" s="3">
+        <v>8.787</v>
+      </c>
+      <c r="V28" s="4">
+        <v>6</v>
+      </c>
+      <c r="W28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C386166.html</t>
         </is>
       </c>
       <c r="X28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C386166.html</t>
-        </is>
-      </c>
-      <c r="Y28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">X7R 50V 1210, AEC-Q200</t>
         </is>
@@ -5151,34 +4956,27 @@
       <c r="Q29" s="3">
         <v>0.0401</v>
       </c>
-      <c r="R29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4010</t>
-        </is>
+      <c r="R29" s="3">
+        <v>0.401</v>
       </c>
       <c r="S29" s="4">
         <v>10</v>
       </c>
-      <c r="T29" s="4">
-        <v>10</v>
-      </c>
-      <c r="U29" s="4">
-        <v>20</v>
-      </c>
-      <c r="V29" s="3">
+      <c r="T29" s="3">
         <v>0.0401</v>
       </c>
-      <c r="W29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8020</t>
-        </is>
-      </c>
-      <c r="X29" s="2" t="inlineStr">
+      <c r="U29" s="3">
+        <v>0.401</v>
+      </c>
+      <c r="V29" s="4">
+        <v>2</v>
+      </c>
+      <c r="W29" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C28323.html</t>
         </is>
       </c>
-      <c r="Y29" s="2"/>
+      <c r="X29" s="2"/>
     </row>
     <row r="30">
       <c r="A30" s="4">
@@ -5252,34 +5050,27 @@
       <c r="Q30" s="3">
         <v>0.0087</v>
       </c>
-      <c r="R30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4350</t>
-        </is>
+      <c r="R30" s="3">
+        <v>0.435</v>
       </c>
       <c r="S30" s="4">
-        <v>20</v>
-      </c>
-      <c r="T30" s="4">
-        <v>30</v>
-      </c>
-      <c r="U30" s="4">
         <v>50</v>
       </c>
-      <c r="V30" s="3">
+      <c r="T30" s="3">
         <v>0.0087</v>
       </c>
-      <c r="W30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4350</t>
+      <c r="U30" s="3">
+        <v>0.435</v>
+      </c>
+      <c r="V30" s="4">
+        <v>4</v>
+      </c>
+      <c r="W30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C14858.html</t>
         </is>
       </c>
       <c r="X30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C14858.html</t>
-        </is>
-      </c>
-      <c r="Y30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package; 100p C0G</t>
         </is>
@@ -5357,34 +5148,27 @@
       <c r="Q31" s="3">
         <v>0.0183</v>
       </c>
-      <c r="R31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.9150</t>
-        </is>
+      <c r="R31" s="3">
+        <v>0.915</v>
       </c>
       <c r="S31" s="4">
-        <v>10</v>
-      </c>
-      <c r="T31" s="4">
-        <v>40</v>
-      </c>
-      <c r="U31" s="4">
         <v>50</v>
       </c>
-      <c r="V31" s="3">
+      <c r="T31" s="3">
         <v>0.0183</v>
       </c>
-      <c r="W31" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.9150</t>
+      <c r="U31" s="3">
+        <v>0.915</v>
+      </c>
+      <c r="V31" s="4">
+        <v>2</v>
+      </c>
+      <c r="W31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C64705.html</t>
         </is>
       </c>
       <c r="X31" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C64705.html</t>
-        </is>
-      </c>
-      <c r="Y31" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -5462,34 +5246,27 @@
       <c r="Q32" s="3">
         <v>0.5519</v>
       </c>
-      <c r="R32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.8633</t>
-        </is>
+      <c r="R32" s="3">
+        <v>3.8633</v>
       </c>
       <c r="S32" s="4">
         <v>35</v>
       </c>
-      <c r="T32" s="4">
-        <v>4</v>
-      </c>
-      <c r="U32" s="4">
-        <v>39</v>
-      </c>
-      <c r="V32" s="3">
+      <c r="T32" s="3">
         <v>0.4156</v>
       </c>
-      <c r="W32" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16.2084</t>
+      <c r="U32" s="3">
+        <v>14.546</v>
+      </c>
+      <c r="V32" s="4">
+        <v>7</v>
+      </c>
+      <c r="W32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C576517.html</t>
         </is>
       </c>
       <c r="X32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C576517.html</t>
-        </is>
-      </c>
-      <c r="Y32" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">X7S 100V 1210; Murata DC-bias chart ~2.60uF at 49 V (model 2.55uF), 25 C</t>
         </is>
@@ -5567,34 +5344,27 @@
       <c r="Q33" s="3">
         <v>0.5157</v>
       </c>
-      <c r="R33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.5157</t>
-        </is>
+      <c r="R33" s="3">
+        <v>0.5157</v>
       </c>
       <c r="S33" s="4">
         <v>5</v>
       </c>
-      <c r="T33" s="4">
-        <v>1</v>
-      </c>
-      <c r="U33" s="4">
-        <v>6</v>
-      </c>
-      <c r="V33" s="3">
+      <c r="T33" s="3">
         <v>0.5157</v>
       </c>
-      <c r="W33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.0942</t>
-        </is>
-      </c>
-      <c r="X33" s="2" t="inlineStr">
+      <c r="U33" s="3">
+        <v>2.5785</v>
+      </c>
+      <c r="V33" s="4">
+        <v>1</v>
+      </c>
+      <c r="W33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C178549.html</t>
         </is>
       </c>
-      <c r="Y33" s="2"/>
+      <c r="X33" s="2"/>
     </row>
     <row r="34">
       <c r="A34" s="4">
@@ -5668,34 +5438,27 @@
       <c r="Q34" s="3">
         <v>0.1312</v>
       </c>
-      <c r="R34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6560</t>
-        </is>
+      <c r="R34" s="3">
+        <v>0.656</v>
       </c>
       <c r="S34" s="4">
         <v>5</v>
       </c>
-      <c r="T34" s="4">
-        <v>5</v>
-      </c>
-      <c r="U34" s="4">
-        <v>10</v>
-      </c>
-      <c r="V34" s="3">
+      <c r="T34" s="3">
         <v>0.1312</v>
       </c>
-      <c r="W34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3120</t>
-        </is>
-      </c>
-      <c r="X34" s="2" t="inlineStr">
+      <c r="U34" s="3">
+        <v>0.656</v>
+      </c>
+      <c r="V34" s="4">
+        <v>1</v>
+      </c>
+      <c r="W34" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C40708.html</t>
         </is>
       </c>
-      <c r="Y34" s="2"/>
+      <c r="X34" s="2"/>
     </row>
     <row r="35">
       <c r="A35" s="4">
@@ -5769,34 +5532,27 @@
       <c r="Q35" s="3">
         <v>0.867</v>
       </c>
-      <c r="R35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8670</t>
-        </is>
+      <c r="R35" s="3">
+        <v>0.867</v>
       </c>
       <c r="S35" s="4">
         <v>5</v>
       </c>
-      <c r="T35" s="4">
-        <v>1</v>
-      </c>
-      <c r="U35" s="4">
-        <v>6</v>
-      </c>
-      <c r="V35" s="3">
+      <c r="T35" s="3">
         <v>0.867</v>
       </c>
-      <c r="W35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5.2020</t>
-        </is>
-      </c>
-      <c r="X35" s="2" t="inlineStr">
+      <c r="U35" s="3">
+        <v>4.335</v>
+      </c>
+      <c r="V35" s="4">
+        <v>1</v>
+      </c>
+      <c r="W35" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C136279.html</t>
         </is>
       </c>
-      <c r="Y35" s="2"/>
+      <c r="X35" s="2"/>
     </row>
     <row r="36">
       <c r="A36" s="4">
@@ -5870,34 +5626,27 @@
       <c r="Q36" s="3">
         <v>0.0031</v>
       </c>
-      <c r="R36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3100</t>
-        </is>
+      <c r="R36" s="3">
+        <v>0.31</v>
       </c>
       <c r="S36" s="4">
-        <v>35</v>
-      </c>
-      <c r="T36" s="4">
-        <v>65</v>
-      </c>
-      <c r="U36" s="4">
         <v>100</v>
       </c>
-      <c r="V36" s="3">
+      <c r="T36" s="3">
         <v>0.0031</v>
       </c>
-      <c r="W36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3100</t>
-        </is>
-      </c>
-      <c r="X36" s="2" t="inlineStr">
+      <c r="U36" s="3">
+        <v>0.31</v>
+      </c>
+      <c r="V36" s="4">
+        <v>7</v>
+      </c>
+      <c r="W36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C25803.html</t>
         </is>
       </c>
-      <c r="Y36" s="2"/>
+      <c r="X36" s="2"/>
     </row>
     <row r="37">
       <c r="A37" s="4">
@@ -5971,34 +5720,27 @@
       <c r="Q37" s="3">
         <v>0.0042</v>
       </c>
-      <c r="R37" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4200</t>
-        </is>
+      <c r="R37" s="3">
+        <v>0.42</v>
       </c>
       <c r="S37" s="4">
-        <v>5</v>
-      </c>
-      <c r="T37" s="4">
-        <v>95</v>
-      </c>
-      <c r="U37" s="4">
         <v>100</v>
       </c>
-      <c r="V37" s="3">
+      <c r="T37" s="3">
         <v>0.0042</v>
       </c>
-      <c r="W37" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4200</t>
+      <c r="U37" s="3">
+        <v>0.42</v>
+      </c>
+      <c r="V37" s="4">
+        <v>1</v>
+      </c>
+      <c r="W37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C31850.html</t>
         </is>
       </c>
       <c r="X37" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C31850.html</t>
-        </is>
-      </c>
-      <c r="Y37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">List price; fetched 2026-09-29 for v0.18 replacement.</t>
         </is>
@@ -6076,34 +5818,27 @@
       <c r="Q38" s="3">
         <v>0.0019</v>
       </c>
-      <c r="R38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.1900</t>
-        </is>
+      <c r="R38" s="3">
+        <v>0.19</v>
       </c>
       <c r="S38" s="4">
-        <v>95</v>
-      </c>
-      <c r="T38" s="4">
-        <v>105</v>
-      </c>
-      <c r="U38" s="4">
-        <v>200</v>
-      </c>
-      <c r="V38" s="3">
+        <v>100</v>
+      </c>
+      <c r="T38" s="3">
         <v>0.0019</v>
       </c>
-      <c r="W38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3800</t>
+      <c r="U38" s="3">
+        <v>0.19</v>
+      </c>
+      <c r="V38" s="4">
+        <v>19</v>
+      </c>
+      <c r="W38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C25804.html</t>
         </is>
       </c>
       <c r="X38" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C25804.html</t>
-        </is>
-      </c>
-      <c r="Y38" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package; 10k 1%</t>
         </is>
@@ -6181,34 +5916,27 @@
       <c r="Q39" s="3">
         <v>0.0026</v>
       </c>
-      <c r="R39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2600</t>
-        </is>
+      <c r="R39" s="3">
+        <v>0.26</v>
       </c>
       <c r="S39" s="4">
-        <v>40</v>
-      </c>
-      <c r="T39" s="4">
-        <v>60</v>
-      </c>
-      <c r="U39" s="4">
         <v>100</v>
       </c>
-      <c r="V39" s="3">
+      <c r="T39" s="3">
         <v>0.0026</v>
       </c>
-      <c r="W39" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2600</t>
+      <c r="U39" s="3">
+        <v>0.26</v>
+      </c>
+      <c r="V39" s="4">
+        <v>8</v>
+      </c>
+      <c r="W39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C21190.html</t>
         </is>
       </c>
       <c r="X39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C21190.html</t>
-        </is>
-      </c>
-      <c r="Y39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1k 1%; R307 RTC battery resistor (v0.20)</t>
         </is>
@@ -6286,34 +6014,27 @@
       <c r="Q40" s="3">
         <v>0.0028</v>
       </c>
-      <c r="R40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2800</t>
-        </is>
+      <c r="R40" s="3">
+        <v>0.28</v>
       </c>
       <c r="S40" s="4">
-        <v>10</v>
-      </c>
-      <c r="T40" s="4">
-        <v>90</v>
-      </c>
-      <c r="U40" s="4">
         <v>100</v>
       </c>
-      <c r="V40" s="3">
+      <c r="T40" s="3">
         <v>0.0028</v>
       </c>
-      <c r="W40" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2800</t>
+      <c r="U40" s="3">
+        <v>0.28</v>
+      </c>
+      <c r="V40" s="4">
+        <v>2</v>
+      </c>
+      <c r="W40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C23162.html</t>
         </is>
       </c>
       <c r="X40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C23162.html</t>
-        </is>
-      </c>
-      <c r="Y40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -6391,34 +6112,27 @@
       <c r="Q41" s="3">
         <v>0.0025</v>
       </c>
-      <c r="R41" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2500</t>
-        </is>
+      <c r="R41" s="3">
+        <v>0.25</v>
       </c>
       <c r="S41" s="4">
-        <v>45</v>
-      </c>
-      <c r="T41" s="4">
-        <v>55</v>
-      </c>
-      <c r="U41" s="4">
         <v>100</v>
       </c>
-      <c r="V41" s="3">
+      <c r="T41" s="3">
         <v>0.0025</v>
       </c>
-      <c r="W41" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2500</t>
+      <c r="U41" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="V41" s="4">
+        <v>9</v>
+      </c>
+      <c r="W41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C23140.html</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C23140.html</t>
-        </is>
-      </c>
-      <c r="Y41" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package; 33R also for the three GPIO gate resistors</t>
         </is>
@@ -6496,34 +6210,27 @@
       <c r="Q42" s="3">
         <v>0.0032</v>
       </c>
-      <c r="R42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.0640</t>
-        </is>
+      <c r="R42" s="3">
+        <v>0.064</v>
       </c>
       <c r="S42" s="4">
-        <v>15</v>
-      </c>
-      <c r="T42" s="4">
-        <v>5</v>
-      </c>
-      <c r="U42" s="4">
         <v>20</v>
       </c>
-      <c r="V42" s="3">
+      <c r="T42" s="3">
         <v>0.0032</v>
       </c>
-      <c r="W42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.0640</t>
+      <c r="U42" s="3">
+        <v>0.064</v>
+      </c>
+      <c r="V42" s="4">
+        <v>3</v>
+      </c>
+      <c r="W42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C22859.html</t>
         </is>
       </c>
       <c r="X42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C22859.html</t>
-        </is>
-      </c>
-      <c r="Y42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -6601,34 +6308,27 @@
       <c r="Q43" s="3">
         <v>0.0031</v>
       </c>
-      <c r="R43" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3100</t>
-        </is>
+      <c r="R43" s="3">
+        <v>0.31</v>
       </c>
       <c r="S43" s="4">
-        <v>15</v>
-      </c>
-      <c r="T43" s="4">
-        <v>85</v>
-      </c>
-      <c r="U43" s="4">
         <v>100</v>
       </c>
-      <c r="V43" s="3">
+      <c r="T43" s="3">
         <v>0.0031</v>
       </c>
-      <c r="W43" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3100</t>
+      <c r="U43" s="3">
+        <v>0.31</v>
+      </c>
+      <c r="V43" s="4">
+        <v>3</v>
+      </c>
+      <c r="W43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C105579.html</t>
         </is>
       </c>
       <c r="X43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C105579.html</t>
-        </is>
-      </c>
-      <c r="Y43" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">R908 MPN from parts review; 47k also for R701-R703</t>
         </is>
@@ -6706,34 +6406,27 @@
       <c r="Q44" s="3">
         <v>0.1011</v>
       </c>
-      <c r="R44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.1011</t>
-        </is>
+      <c r="R44" s="3">
+        <v>0.1011</v>
       </c>
       <c r="S44" s="4">
         <v>5</v>
       </c>
-      <c r="T44" s="4">
-        <v>1</v>
-      </c>
-      <c r="U44" s="4">
-        <v>6</v>
-      </c>
-      <c r="V44" s="3">
+      <c r="T44" s="3">
         <v>0.1011</v>
       </c>
-      <c r="W44" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6066</t>
-        </is>
-      </c>
-      <c r="X44" s="2" t="inlineStr">
+      <c r="U44" s="3">
+        <v>0.5055</v>
+      </c>
+      <c r="V44" s="4">
+        <v>1</v>
+      </c>
+      <c r="W44" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C19633795.html</t>
         </is>
       </c>
-      <c r="Y44" s="2"/>
+      <c r="X44" s="2"/>
     </row>
     <row r="45">
       <c r="A45" s="4">
@@ -6807,34 +6500,27 @@
       <c r="Q45" s="3">
         <v>0.0722</v>
       </c>
-      <c r="R45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7220</t>
-        </is>
+      <c r="R45" s="3">
+        <v>0.722</v>
       </c>
       <c r="S45" s="4">
-        <v>5</v>
-      </c>
-      <c r="T45" s="4">
-        <v>5</v>
-      </c>
-      <c r="U45" s="4">
         <v>10</v>
       </c>
-      <c r="V45" s="3">
+      <c r="T45" s="3">
         <v>0.0722</v>
       </c>
-      <c r="W45" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.7220</t>
+      <c r="U45" s="3">
+        <v>0.722</v>
+      </c>
+      <c r="V45" s="4">
+        <v>1</v>
+      </c>
+      <c r="W45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C48533605.html</t>
         </is>
       </c>
       <c r="X45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C48533605.html</t>
-        </is>
-      </c>
-      <c r="Y45" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">0.18 ohm option B selected since v0.17; same fitted shunt retained.</t>
         </is>
@@ -6912,34 +6598,27 @@
       <c r="Q46" s="3">
         <v>0.0025</v>
       </c>
-      <c r="R46" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2500</t>
-        </is>
+      <c r="R46" s="3">
+        <v>0.25</v>
       </c>
       <c r="S46" s="4">
-        <v>10</v>
-      </c>
-      <c r="T46" s="4">
-        <v>90</v>
-      </c>
-      <c r="U46" s="4">
         <v>100</v>
       </c>
-      <c r="V46" s="3">
+      <c r="T46" s="3">
         <v>0.0025</v>
       </c>
-      <c r="W46" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.2500</t>
+      <c r="U46" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="V46" s="4">
+        <v>2</v>
+      </c>
+      <c r="W46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C25814.html</t>
         </is>
       </c>
       <c r="X46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C25814.html</t>
-        </is>
-      </c>
-      <c r="Y46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -7017,34 +6696,27 @@
       <c r="Q47" s="3">
         <v>0.0033</v>
       </c>
-      <c r="R47" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3300</t>
-        </is>
+      <c r="R47" s="3">
+        <v>0.33</v>
       </c>
       <c r="S47" s="4">
-        <v>5</v>
-      </c>
-      <c r="T47" s="4">
-        <v>95</v>
-      </c>
-      <c r="U47" s="4">
         <v>100</v>
       </c>
-      <c r="V47" s="3">
+      <c r="T47" s="3">
         <v>0.0033</v>
       </c>
-      <c r="W47" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.3300</t>
+      <c r="U47" s="3">
+        <v>0.33</v>
+      </c>
+      <c r="V47" s="4">
+        <v>1</v>
+      </c>
+      <c r="W47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C13167.html</t>
         </is>
       </c>
       <c r="X47" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C13167.html</t>
-        </is>
-      </c>
-      <c r="Y47" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -7122,34 +6794,27 @@
       <c r="Q48" s="3">
         <v>0.0495</v>
       </c>
-      <c r="R48" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4950</t>
-        </is>
+      <c r="R48" s="3">
+        <v>0.495</v>
       </c>
       <c r="S48" s="4">
-        <v>5</v>
-      </c>
-      <c r="T48" s="4">
-        <v>5</v>
-      </c>
-      <c r="U48" s="4">
         <v>10</v>
       </c>
-      <c r="V48" s="3">
+      <c r="T48" s="3">
         <v>0.0495</v>
       </c>
-      <c r="W48" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4950</t>
-        </is>
-      </c>
-      <c r="X48" s="2" t="inlineStr">
+      <c r="U48" s="3">
+        <v>0.495</v>
+      </c>
+      <c r="V48" s="4">
+        <v>1</v>
+      </c>
+      <c r="W48" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C52015951.html</t>
         </is>
       </c>
-      <c r="Y48" s="2"/>
+      <c r="X48" s="2"/>
     </row>
     <row r="49">
       <c r="A49" s="4">
@@ -7223,34 +6888,27 @@
       <c r="Q49" s="3">
         <v>0.027</v>
       </c>
-      <c r="R49" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.5400</t>
-        </is>
+      <c r="R49" s="3">
+        <v>0.54</v>
       </c>
       <c r="S49" s="4">
-        <v>5</v>
-      </c>
-      <c r="T49" s="4">
-        <v>15</v>
-      </c>
-      <c r="U49" s="4">
         <v>20</v>
       </c>
-      <c r="V49" s="3">
+      <c r="T49" s="3">
         <v>0.027</v>
       </c>
-      <c r="W49" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.5400</t>
-        </is>
-      </c>
-      <c r="X49" s="2" t="inlineStr">
+      <c r="U49" s="3">
+        <v>0.54</v>
+      </c>
+      <c r="V49" s="4">
+        <v>1</v>
+      </c>
+      <c r="W49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C22464907.html</t>
         </is>
       </c>
-      <c r="Y49" s="2"/>
+      <c r="X49" s="2"/>
     </row>
     <row r="50">
       <c r="A50" s="4">
@@ -7324,34 +6982,27 @@
       <c r="Q50" s="3">
         <v>0.0437</v>
       </c>
-      <c r="R50" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8740</t>
-        </is>
+      <c r="R50" s="3">
+        <v>0.874</v>
       </c>
       <c r="S50" s="4">
-        <v>5</v>
-      </c>
-      <c r="T50" s="4">
-        <v>15</v>
-      </c>
-      <c r="U50" s="4">
         <v>20</v>
       </c>
-      <c r="V50" s="3">
+      <c r="T50" s="3">
         <v>0.0437</v>
       </c>
-      <c r="W50" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8740</t>
-        </is>
-      </c>
-      <c r="X50" s="2" t="inlineStr">
+      <c r="U50" s="3">
+        <v>0.874</v>
+      </c>
+      <c r="V50" s="4">
+        <v>1</v>
+      </c>
+      <c r="W50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C326734.html</t>
         </is>
       </c>
-      <c r="Y50" s="2"/>
+      <c r="X50" s="2"/>
     </row>
     <row r="51">
       <c r="A51" s="4">
@@ -7425,34 +7076,27 @@
       <c r="Q51" s="3">
         <v>0.033</v>
       </c>
-      <c r="R51" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6600</t>
-        </is>
+      <c r="R51" s="3">
+        <v>0.66</v>
       </c>
       <c r="S51" s="4">
-        <v>5</v>
-      </c>
-      <c r="T51" s="4">
-        <v>15</v>
-      </c>
-      <c r="U51" s="4">
         <v>20</v>
       </c>
-      <c r="V51" s="3">
+      <c r="T51" s="3">
         <v>0.033</v>
       </c>
-      <c r="W51" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6600</t>
-        </is>
-      </c>
-      <c r="X51" s="2" t="inlineStr">
+      <c r="U51" s="3">
+        <v>0.66</v>
+      </c>
+      <c r="V51" s="4">
+        <v>1</v>
+      </c>
+      <c r="W51" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C95204.html</t>
         </is>
       </c>
-      <c r="Y51" s="2"/>
+      <c r="X51" s="2"/>
     </row>
     <row r="52">
       <c r="A52" s="4">
@@ -7526,34 +7170,27 @@
       <c r="Q52" s="3">
         <v>0.0015</v>
       </c>
-      <c r="R52" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.1500</t>
-        </is>
+      <c r="R52" s="3">
+        <v>0.15</v>
       </c>
       <c r="S52" s="4">
-        <v>5</v>
-      </c>
-      <c r="T52" s="4">
-        <v>95</v>
-      </c>
-      <c r="U52" s="4">
         <v>100</v>
       </c>
-      <c r="V52" s="3">
+      <c r="T52" s="3">
         <v>0.0015</v>
       </c>
-      <c r="W52" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.1500</t>
-        </is>
-      </c>
-      <c r="X52" s="2" t="inlineStr">
+      <c r="U52" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="V52" s="4">
+        <v>1</v>
+      </c>
+      <c r="W52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C23203.html</t>
         </is>
       </c>
-      <c r="Y52" s="2"/>
+      <c r="X52" s="2"/>
     </row>
     <row r="53">
       <c r="A53" s="4">
@@ -7627,34 +7264,27 @@
       <c r="Q53" s="3">
         <v>0.0307</v>
       </c>
-      <c r="R53" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6140</t>
-        </is>
+      <c r="R53" s="3">
+        <v>0.614</v>
       </c>
       <c r="S53" s="4">
-        <v>5</v>
-      </c>
-      <c r="T53" s="4">
-        <v>15</v>
-      </c>
-      <c r="U53" s="4">
         <v>20</v>
       </c>
-      <c r="V53" s="3">
+      <c r="T53" s="3">
         <v>0.0307</v>
       </c>
-      <c r="W53" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6140</t>
+      <c r="U53" s="3">
+        <v>0.614</v>
+      </c>
+      <c r="V53" s="4">
+        <v>1</v>
+      </c>
+      <c r="W53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C70065.html</t>
         </is>
       </c>
       <c r="X53" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C70065.html</t>
-        </is>
-      </c>
-      <c r="Y53" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package; PTC 100mA 60V 1206</t>
         </is>
@@ -7732,34 +7362,27 @@
       <c r="Q54" s="3">
         <v>0.2536</v>
       </c>
-      <c r="R54" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2680</t>
-        </is>
+      <c r="R54" s="3">
+        <v>1.268</v>
       </c>
       <c r="S54" s="4">
         <v>15</v>
       </c>
-      <c r="T54" s="4">
-        <v>5</v>
-      </c>
-      <c r="U54" s="4">
-        <v>20</v>
-      </c>
-      <c r="V54" s="3">
+      <c r="T54" s="3">
         <v>0.2536</v>
       </c>
-      <c r="W54" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5.0720</t>
-        </is>
-      </c>
-      <c r="X54" s="2" t="inlineStr">
+      <c r="U54" s="3">
+        <v>3.804</v>
+      </c>
+      <c r="V54" s="4">
+        <v>3</v>
+      </c>
+      <c r="W54" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C3099.html</t>
         </is>
       </c>
-      <c r="Y54" s="2"/>
+      <c r="X54" s="2"/>
     </row>
     <row r="55">
       <c r="A55" s="4">
@@ -7833,34 +7456,27 @@
       <c r="Q55" s="3">
         <v>0.2477</v>
       </c>
-      <c r="R55" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2385</t>
-        </is>
+      <c r="R55" s="3">
+        <v>1.2385</v>
       </c>
       <c r="S55" s="4">
         <v>5</v>
       </c>
-      <c r="T55" s="4">
-        <v>5</v>
-      </c>
-      <c r="U55" s="4">
-        <v>10</v>
-      </c>
-      <c r="V55" s="3">
+      <c r="T55" s="3">
         <v>0.2477</v>
       </c>
-      <c r="W55" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.4770</t>
-        </is>
-      </c>
-      <c r="X55" s="2" t="inlineStr">
+      <c r="U55" s="3">
+        <v>1.2385</v>
+      </c>
+      <c r="V55" s="4">
+        <v>1</v>
+      </c>
+      <c r="W55" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C178982.html</t>
         </is>
       </c>
-      <c r="Y55" s="2"/>
+      <c r="X55" s="2"/>
     </row>
     <row r="56">
       <c r="A56" s="4">
@@ -7934,34 +7550,27 @@
       <c r="Q56" s="3">
         <v>0.2556</v>
       </c>
-      <c r="R56" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2780</t>
-        </is>
+      <c r="R56" s="3">
+        <v>1.278</v>
       </c>
       <c r="S56" s="4">
         <v>10</v>
       </c>
-      <c r="T56" s="4">
-        <v>5</v>
-      </c>
-      <c r="U56" s="4">
-        <v>15</v>
-      </c>
-      <c r="V56" s="3">
+      <c r="T56" s="3">
         <v>0.2556</v>
       </c>
-      <c r="W56" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.8340</t>
+      <c r="U56" s="3">
+        <v>2.556</v>
+      </c>
+      <c r="V56" s="4">
+        <v>2</v>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C13982.html</t>
         </is>
       </c>
       <c r="X56" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C13982.html</t>
-        </is>
-      </c>
-      <c r="Y56" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">F904 raised from 2A to 3A to share the F721 part</t>
         </is>
@@ -8039,34 +7648,27 @@
       <c r="Q57" s="3">
         <v>0.2775</v>
       </c>
-      <c r="R57" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.3875</t>
-        </is>
+      <c r="R57" s="3">
+        <v>1.3875</v>
       </c>
       <c r="S57" s="4">
         <v>5</v>
       </c>
-      <c r="T57" s="4">
-        <v>5</v>
-      </c>
-      <c r="U57" s="4">
-        <v>10</v>
-      </c>
-      <c r="V57" s="3">
+      <c r="T57" s="3">
         <v>0.2775</v>
       </c>
-      <c r="W57" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.7750</t>
+      <c r="U57" s="3">
+        <v>1.3875</v>
+      </c>
+      <c r="V57" s="4">
+        <v>1</v>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C19727305.html</t>
         </is>
       </c>
       <c r="X57" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C19727305.html</t>
-        </is>
-      </c>
-      <c r="Y57" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">holder only</t>
         </is>
@@ -8144,34 +7746,27 @@
       <c r="Q58" s="3">
         <v>0.0419</v>
       </c>
-      <c r="R58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4190</t>
-        </is>
+      <c r="R58" s="3">
+        <v>0.419</v>
       </c>
       <c r="S58" s="4">
-        <v>5</v>
-      </c>
-      <c r="T58" s="4">
-        <v>5</v>
-      </c>
-      <c r="U58" s="4">
         <v>10</v>
       </c>
-      <c r="V58" s="3">
+      <c r="T58" s="3">
         <v>0.0419</v>
       </c>
-      <c r="W58" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4190</t>
+      <c r="U58" s="3">
+        <v>0.419</v>
+      </c>
+      <c r="V58" s="4">
+        <v>1</v>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C37208.html</t>
         </is>
       </c>
       <c r="X58" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C37208.html</t>
-        </is>
-      </c>
-      <c r="Y58" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -8249,34 +7844,27 @@
       <c r="Q59" s="3">
         <v>0.0622</v>
       </c>
-      <c r="R59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6220</t>
-        </is>
+      <c r="R59" s="3">
+        <v>0.622</v>
       </c>
       <c r="S59" s="4">
-        <v>5</v>
-      </c>
-      <c r="T59" s="4">
-        <v>5</v>
-      </c>
-      <c r="U59" s="4">
         <v>10</v>
       </c>
-      <c r="V59" s="3">
+      <c r="T59" s="3">
         <v>0.0622</v>
       </c>
-      <c r="W59" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6220</t>
+      <c r="U59" s="3">
+        <v>0.622</v>
+      </c>
+      <c r="V59" s="4">
+        <v>1</v>
+      </c>
+      <c r="W59" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C144395.html</t>
         </is>
       </c>
       <c r="X59" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C144395.html</t>
-        </is>
-      </c>
-      <c r="Y59" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">equivalent allowed: representative LCSC part for this value and package</t>
         </is>
@@ -8354,34 +7942,27 @@
       <c r="Q60" s="3">
         <v>0.1832</v>
       </c>
-      <c r="R60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.9160</t>
-        </is>
+      <c r="R60" s="3">
+        <v>0.916</v>
       </c>
       <c r="S60" s="4">
         <v>15</v>
       </c>
-      <c r="T60" s="4">
-        <v>5</v>
-      </c>
-      <c r="U60" s="4">
-        <v>20</v>
-      </c>
-      <c r="V60" s="3">
+      <c r="T60" s="3">
         <v>0.1832</v>
       </c>
-      <c r="W60" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.6640</t>
-        </is>
-      </c>
-      <c r="X60" s="2" t="inlineStr">
+      <c r="U60" s="3">
+        <v>2.748</v>
+      </c>
+      <c r="V60" s="4">
+        <v>3</v>
+      </c>
+      <c r="W60" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C466970.html</t>
         </is>
       </c>
-      <c r="Y60" s="2"/>
+      <c r="X60" s="2"/>
     </row>
     <row r="61">
       <c r="A61" s="4">
@@ -8455,34 +8036,27 @@
       <c r="Q61" s="3">
         <v>0.1937</v>
       </c>
-      <c r="R61" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.9685</t>
-        </is>
+      <c r="R61" s="3">
+        <v>0.9685</v>
       </c>
       <c r="S61" s="4">
         <v>5</v>
       </c>
-      <c r="T61" s="4">
-        <v>5</v>
-      </c>
-      <c r="U61" s="4">
-        <v>10</v>
-      </c>
-      <c r="V61" s="3">
+      <c r="T61" s="3">
         <v>0.1937</v>
       </c>
-      <c r="W61" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.9370</t>
+      <c r="U61" s="3">
+        <v>0.9685</v>
+      </c>
+      <c r="V61" s="4">
+        <v>1</v>
+      </c>
+      <c r="W61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C91145.html</t>
         </is>
       </c>
       <c r="X61" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C91145.html</t>
-        </is>
-      </c>
-      <c r="Y61" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">push-push microSD, card detect unused; list price (8 % promotion ignored)</t>
         </is>
@@ -8560,34 +8134,27 @@
       <c r="Q62" s="3">
         <v>0.4026</v>
       </c>
-      <c r="R62" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.0130</t>
-        </is>
+      <c r="R62" s="3">
+        <v>2.013</v>
       </c>
       <c r="S62" s="4">
         <v>10</v>
       </c>
-      <c r="T62" s="4">
-        <v>5</v>
-      </c>
-      <c r="U62" s="4">
-        <v>15</v>
-      </c>
-      <c r="V62" s="3">
+      <c r="T62" s="3">
         <v>0.4026</v>
       </c>
-      <c r="W62" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6.0390</t>
-        </is>
-      </c>
-      <c r="X62" s="2" t="inlineStr">
+      <c r="U62" s="3">
+        <v>4.026</v>
+      </c>
+      <c r="V62" s="4">
+        <v>2</v>
+      </c>
+      <c r="W62" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C2757925.html</t>
         </is>
       </c>
-      <c r="Y62" s="2"/>
+      <c r="X62" s="2"/>
     </row>
     <row r="63">
       <c r="A63" s="4">
@@ -8661,34 +8228,27 @@
       <c r="Q63" s="3">
         <v>0.1349</v>
       </c>
-      <c r="R63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6745</t>
-        </is>
+      <c r="R63" s="3">
+        <v>0.6745</v>
       </c>
       <c r="S63" s="4">
         <v>15</v>
       </c>
-      <c r="T63" s="4">
-        <v>5</v>
-      </c>
-      <c r="U63" s="4">
-        <v>20</v>
-      </c>
-      <c r="V63" s="3">
+      <c r="T63" s="3">
         <v>0.1349</v>
       </c>
-      <c r="W63" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2.6980</t>
-        </is>
-      </c>
-      <c r="X63" s="2" t="inlineStr">
+      <c r="U63" s="3">
+        <v>2.0235</v>
+      </c>
+      <c r="V63" s="4">
+        <v>3</v>
+      </c>
+      <c r="W63" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C8465.html</t>
         </is>
       </c>
-      <c r="Y63" s="2"/>
+      <c r="X63" s="2"/>
     </row>
     <row r="64">
       <c r="A64" s="4">
@@ -8762,34 +8322,25 @@
       <c r="Q64" s="3">
         <v>0.6072</v>
       </c>
-      <c r="R64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6072</t>
-        </is>
+      <c r="R64" s="3">
+        <v>0.6072</v>
       </c>
       <c r="S64" s="4">
         <v>5</v>
       </c>
-      <c r="T64" s="4">
-        <v>1</v>
-      </c>
-      <c r="U64" s="4">
-        <v>6</v>
-      </c>
-      <c r="V64" s="3">
+      <c r="T64" s="3">
         <v>0.6072</v>
       </c>
-      <c r="W64" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.6432</t>
+      <c r="U64" s="3">
+        <v>3.036</v>
+      </c>
+      <c r="V64" s="2"/>
+      <c r="W64" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C98732.html</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C98732.html</t>
-        </is>
-      </c>
-      <c r="Y64" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">0 in stock at LCSC; buy elsewhere; JLCPCB parts library lists 8708 in stock (assembly service)</t>
         </is>
@@ -8867,34 +8418,27 @@
       <c r="Q65" s="3">
         <v>0.0207</v>
       </c>
-      <c r="R65" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4140</t>
-        </is>
+      <c r="R65" s="3">
+        <v>0.414</v>
       </c>
       <c r="S65" s="4">
-        <v>10</v>
-      </c>
-      <c r="T65" s="4">
-        <v>10</v>
-      </c>
-      <c r="U65" s="4">
         <v>20</v>
       </c>
-      <c r="V65" s="3">
+      <c r="T65" s="3">
         <v>0.0207</v>
       </c>
-      <c r="W65" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.4140</t>
-        </is>
-      </c>
-      <c r="X65" s="2" t="inlineStr">
+      <c r="U65" s="3">
+        <v>0.414</v>
+      </c>
+      <c r="V65" s="4">
+        <v>2</v>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C318884.html</t>
         </is>
       </c>
-      <c r="Y65" s="2"/>
+      <c r="X65" s="2"/>
     </row>
     <row r="66">
       <c r="A66" s="4">
@@ -8968,34 +8512,27 @@
       <c r="Q66" s="3">
         <v>0.3983</v>
       </c>
-      <c r="R66" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.9915</t>
-        </is>
+      <c r="R66" s="3">
+        <v>1.9915</v>
       </c>
       <c r="S66" s="4">
         <v>5</v>
       </c>
-      <c r="T66" s="4">
-        <v>5</v>
-      </c>
-      <c r="U66" s="4">
-        <v>10</v>
-      </c>
-      <c r="V66" s="3">
+      <c r="T66" s="3">
         <v>0.3983</v>
       </c>
-      <c r="W66" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3.9830</t>
+      <c r="U66" s="3">
+        <v>1.9915</v>
+      </c>
+      <c r="V66" s="4">
+        <v>1</v>
+      </c>
+      <c r="W66" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lcsc.com/product-detail/C2979167.html</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.lcsc.com/product-detail/C2979167.html</t>
-        </is>
-      </c>
-      <c r="Y66" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">holder only; mounted on the bottom side</t>
         </is>
@@ -9073,34 +8610,27 @@
       <c r="Q67" s="3">
         <v>0.1733</v>
       </c>
-      <c r="R67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.8665</t>
-        </is>
+      <c r="R67" s="3">
+        <v>0.8665</v>
       </c>
       <c r="S67" s="4">
         <v>5</v>
       </c>
-      <c r="T67" s="4">
-        <v>5</v>
-      </c>
-      <c r="U67" s="4">
-        <v>10</v>
-      </c>
-      <c r="V67" s="3">
+      <c r="T67" s="3">
         <v>0.1733</v>
       </c>
-      <c r="W67" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.7330</t>
-        </is>
-      </c>
-      <c r="X67" s="2" t="inlineStr">
+      <c r="U67" s="3">
+        <v>0.8665</v>
+      </c>
+      <c r="V67" s="4">
+        <v>1</v>
+      </c>
+      <c r="W67" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C32346.html</t>
         </is>
       </c>
-      <c r="Y67" s="2"/>
+      <c r="X67" s="2"/>
     </row>
     <row r="68">
       <c r="A68" s="4">
@@ -9154,8 +8684,7 @@
       <c r="U68" s="2"/>
       <c r="V68" s="2"/>
       <c r="W68" s="2"/>
-      <c r="X68" s="2"/>
-      <c r="Y68" s="2" t="inlineStr">
+      <c r="X68" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">no CR2032 cell found at LCSC on the snapshot date; buy locally</t>
         </is>
@@ -9225,34 +8754,27 @@
       <c r="Q69" s="3">
         <v>0.1236</v>
       </c>
-      <c r="R69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.6180</t>
-        </is>
+      <c r="R69" s="3">
+        <v>0.618</v>
       </c>
       <c r="S69" s="4">
         <v>5</v>
       </c>
-      <c r="T69" s="4">
-        <v>5</v>
-      </c>
-      <c r="U69" s="4">
-        <v>10</v>
-      </c>
-      <c r="V69" s="3">
+      <c r="T69" s="3">
         <v>0.1236</v>
       </c>
-      <c r="W69" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1.2360</t>
-        </is>
-      </c>
-      <c r="X69" s="2" t="inlineStr">
+      <c r="U69" s="3">
+        <v>0.618</v>
+      </c>
+      <c r="V69" s="4">
+        <v>1</v>
+      </c>
+      <c r="W69" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">https://www.lcsc.com/product-detail/C151094.html</t>
         </is>
       </c>
-      <c r="Y69" s="2"/>
+      <c r="X69" s="2"/>
     </row>
     <row r="70">
       <c r="A70" s="7">
@@ -9306,8 +8828,7 @@
       <c r="U70" s="7"/>
       <c r="V70" s="7"/>
       <c r="W70" s="7"/>
-      <c r="X70" s="7"/>
-      <c r="Y70" s="7" t="inlineStr">
+      <c r="X70" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">not fitted</t>
         </is>
@@ -9365,8 +8886,7 @@
       <c r="U71" s="7"/>
       <c r="V71" s="7"/>
       <c r="W71" s="7"/>
-      <c r="X71" s="7"/>
-      <c r="Y71" s="7" t="inlineStr">
+      <c r="X71" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">copper only: Kelvin taps at the LED-driver shunts</t>
         </is>
@@ -9424,15 +8944,14 @@
       <c r="U72" s="7"/>
       <c r="V72" s="7"/>
       <c r="W72" s="7"/>
-      <c r="X72" s="7"/>
-      <c r="Y72" s="7" t="inlineStr">
+      <c r="X72" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">copper pad only</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y72"/>
+  <autoFilter ref="A1:X72"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
@@ -9492,12 +9011,12 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build</t>
+          <t xml:space="preserve">Upload file</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 boards; quantities include spares (10 %, at least one piece) and the LCSC minimum/multiple</t>
+          <t xml:space="preserve">quantities for 1 board(s), spares 0 %, not rounded to the LCSC minimum order</t>
         </is>
       </c>
     </row>
@@ -9542,7 +9061,7 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order for 1 board, no spares</t>
+          <t xml:space="preserve">Order for 1 board</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
@@ -9554,7 +9073,7 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order for 5 boards, no spares</t>
+          <t xml:space="preserve">Order for 5 boards</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
@@ -9566,12 +9085,12 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Order for 5 boards, with spares (upload file)</t>
+          <t xml:space="preserve">Upload file after LCSC minimum orders</t>
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">188.2771</t>
+          <t xml:space="preserve">59.9157</t>
         </is>
       </c>
     </row>

</xml_diff>